<commit_message>
Updated the Measures excel file
</commit_message>
<xml_diff>
--- a/Global_Markets_Pulse_Measures/Global_Markets_Pulse_Measures.xlsx
+++ b/Global_Markets_Pulse_Measures/Global_Markets_Pulse_Measures.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\GVX0EPF00008594\EXCELCNV\967abb45-2a50-4236-bcbb-122c0a62eb76\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B01E5D01-688F-4018-AD3F-D0DE95C8AFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{825E76D4-38CC-4879-BFCA-AE658B0C6728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{BFC91BB5-B084-49E1-B128-C723D056B03D}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" activeTab="2" xr2:uid="{BFC91BB5-B084-49E1-B128-C723D056B03D}"/>
   </bookViews>
   <sheets>
-    <sheet name="in" sheetId="1" r:id="rId1"/>
+    <sheet name="Performance" sheetId="1" r:id="rId1"/>
+    <sheet name="Volatility" sheetId="2" r:id="rId2"/>
+    <sheet name="Risk" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="247">
   <si>
     <t>Type of Measure</t>
   </si>
@@ -3979,21 +3981,759 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="409.6">
+    <row r="30" spans="1:5">
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="3:3">
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="3:3">
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="3:3">
+      <c r="C37" s="2"/>
+    </row>
+    <row r="38" spans="3:3">
+      <c r="C38" s="2"/>
+    </row>
+    <row r="39" spans="3:3">
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" spans="3:3">
+      <c r="C40" s="2"/>
+    </row>
+    <row r="41" spans="3:3">
+      <c r="C41" s="2"/>
+    </row>
+    <row r="42" spans="3:3">
+      <c r="C42" s="2"/>
+    </row>
+    <row r="43" spans="3:3">
+      <c r="C43" s="2"/>
+    </row>
+    <row r="44" spans="3:3">
+      <c r="C44" s="2"/>
+    </row>
+    <row r="45" spans="3:3">
+      <c r="C45" s="2"/>
+    </row>
+    <row r="46" spans="3:3">
+      <c r="C46" s="2"/>
+    </row>
+    <row r="47" spans="3:3">
+      <c r="C47" s="2"/>
+    </row>
+    <row r="48" spans="3:3">
+      <c r="C48" s="2"/>
+    </row>
+    <row r="49" spans="3:3">
+      <c r="C49" s="2"/>
+    </row>
+    <row r="50" spans="3:3">
+      <c r="C50" s="2"/>
+    </row>
+    <row r="51" spans="3:3">
+      <c r="C51" s="2"/>
+    </row>
+    <row r="52" spans="3:3">
+      <c r="C52" s="2"/>
+    </row>
+    <row r="53" spans="3:3">
+      <c r="C53" s="2"/>
+    </row>
+    <row r="54" spans="3:3">
+      <c r="C54" s="2"/>
+    </row>
+    <row r="55" spans="3:3">
+      <c r="C55" s="2"/>
+    </row>
+    <row r="56" spans="3:3">
+      <c r="C56" s="2"/>
+    </row>
+    <row r="57" spans="3:3">
+      <c r="C57" s="2"/>
+    </row>
+    <row r="58" spans="3:3">
+      <c r="C58" s="2"/>
+    </row>
+    <row r="59" spans="3:3">
+      <c r="C59" s="2"/>
+    </row>
+    <row r="60" spans="3:3">
+      <c r="C60" s="2"/>
+    </row>
+    <row r="61" spans="3:3">
+      <c r="C61" s="2"/>
+    </row>
+    <row r="62" spans="3:3">
+      <c r="C62" s="2"/>
+    </row>
+    <row r="63" spans="3:3">
+      <c r="C63" s="2"/>
+    </row>
+    <row r="64" spans="3:3">
+      <c r="C64" s="2"/>
+    </row>
+    <row r="65" spans="3:3">
+      <c r="C65" s="2"/>
+    </row>
+    <row r="66" spans="3:3">
+      <c r="C66" s="2"/>
+    </row>
+    <row r="67" spans="3:3">
+      <c r="C67" s="2"/>
+    </row>
+    <row r="68" spans="3:3">
+      <c r="C68" s="2"/>
+    </row>
+    <row r="69" spans="3:3">
+      <c r="C69" s="2"/>
+    </row>
+    <row r="70" spans="3:3">
+      <c r="C70" s="2"/>
+    </row>
+    <row r="71" spans="3:3">
+      <c r="C71" s="2"/>
+    </row>
+    <row r="72" spans="3:3">
+      <c r="C72" s="2"/>
+    </row>
+    <row r="73" spans="3:3">
+      <c r="C73" s="2"/>
+    </row>
+    <row r="74" spans="3:3">
+      <c r="C74" s="2"/>
+    </row>
+    <row r="75" spans="3:3">
+      <c r="C75" s="2"/>
+    </row>
+    <row r="76" spans="3:3">
+      <c r="C76" s="2"/>
+    </row>
+    <row r="77" spans="3:3">
+      <c r="C77" s="2"/>
+    </row>
+    <row r="78" spans="3:3">
+      <c r="C78" s="2"/>
+    </row>
+    <row r="79" spans="3:3">
+      <c r="C79" s="2"/>
+    </row>
+    <row r="80" spans="3:3">
+      <c r="C80" s="2"/>
+    </row>
+    <row r="81" spans="3:3">
+      <c r="C81" s="2"/>
+    </row>
+    <row r="82" spans="3:3">
+      <c r="C82" s="2"/>
+    </row>
+    <row r="83" spans="3:3">
+      <c r="C83" s="2"/>
+    </row>
+    <row r="84" spans="3:3">
+      <c r="C84" s="2"/>
+    </row>
+    <row r="85" spans="3:3">
+      <c r="C85" s="2"/>
+    </row>
+    <row r="86" spans="3:3">
+      <c r="C86" s="2"/>
+    </row>
+    <row r="87" spans="3:3">
+      <c r="C87" s="2"/>
+    </row>
+    <row r="88" spans="3:3">
+      <c r="C88" s="2"/>
+    </row>
+    <row r="89" spans="3:3">
+      <c r="C89" s="2"/>
+    </row>
+    <row r="90" spans="3:3">
+      <c r="C90" s="2"/>
+    </row>
+    <row r="91" spans="3:3">
+      <c r="C91" s="2"/>
+    </row>
+    <row r="92" spans="3:3">
+      <c r="C92" s="2"/>
+    </row>
+    <row r="93" spans="3:3">
+      <c r="C93" s="2"/>
+    </row>
+    <row r="94" spans="3:3">
+      <c r="C94" s="2"/>
+    </row>
+    <row r="95" spans="3:3">
+      <c r="C95" s="2"/>
+    </row>
+    <row r="96" spans="3:3">
+      <c r="C96" s="2"/>
+    </row>
+    <row r="97" spans="3:3">
+      <c r="C97" s="2"/>
+    </row>
+    <row r="98" spans="3:3">
+      <c r="C98" s="2"/>
+    </row>
+    <row r="99" spans="3:3">
+      <c r="C99" s="2"/>
+    </row>
+    <row r="100" spans="3:3">
+      <c r="C100" s="2"/>
+    </row>
+    <row r="101" spans="3:3">
+      <c r="C101" s="2"/>
+    </row>
+    <row r="102" spans="3:3">
+      <c r="C102" s="2"/>
+    </row>
+    <row r="103" spans="3:3">
+      <c r="C103" s="2"/>
+    </row>
+    <row r="104" spans="3:3">
+      <c r="C104" s="2"/>
+    </row>
+    <row r="105" spans="3:3">
+      <c r="C105" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8EAEF6F-D486-4479-BEBA-925B59B54109}">
+  <dimension ref="A1:E77"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="5" max="5" width="47.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="409.6">
+      <c r="A2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.6">
+      <c r="A3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="137.25">
+      <c r="A4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="321">
+      <c r="A5" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="137.25">
+      <c r="A6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="259.5">
+      <c r="A7" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="229.5">
+      <c r="A8" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="259.5">
+      <c r="A9" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="183">
+      <c r="A10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="259.5">
+      <c r="A11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="183">
+      <c r="A12" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="290.25">
+      <c r="A13" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="409.6">
+      <c r="A14" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="137.25">
+      <c r="A15" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="259.5">
+      <c r="A16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="198">
+      <c r="A17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="259.5">
+      <c r="A18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="106.5">
+      <c r="A19" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="106.5">
+      <c r="A20" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="76.5">
+      <c r="A21" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="259.5">
+      <c r="A22" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="106.5">
+      <c r="A23" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="106.5">
+      <c r="A24" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="351">
+      <c r="A25" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="213">
+      <c r="A26" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="213">
+      <c r="A27" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="167.25">
+      <c r="A28" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="106.5">
+      <c r="A29" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="275.25">
       <c r="A30" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>74</v>
+        <v>139</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>76</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="409.6">
@@ -4004,135 +4744,135 @@
         <v>77</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>78</v>
+        <v>142</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="137.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="259.5">
       <c r="A32" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>81</v>
+        <v>144</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="321">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="183">
       <c r="A33" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>83</v>
+        <v>146</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>84</v>
+        <v>147</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="137.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="183">
       <c r="A34" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>80</v>
+        <v>146</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>86</v>
+        <v>149</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="259.5">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="198">
       <c r="A35" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>89</v>
+        <v>151</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="229.5">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="106.5">
       <c r="A36" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>92</v>
+        <v>153</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>41</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="259.5">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="409.6">
       <c r="A37" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>91</v>
+        <v>155</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>94</v>
+        <v>156</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="183">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="409.6">
       <c r="A38" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>91</v>
+        <v>155</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>96</v>
+        <v>158</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="259.5">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="229.5">
       <c r="A39" s="3" t="s">
         <v>72</v>
       </c>
@@ -4140,16 +4880,16 @@
         <v>91</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>98</v>
+        <v>160</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="183">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="259.5">
       <c r="A40" s="3" t="s">
         <v>72</v>
       </c>
@@ -4157,30 +4897,30 @@
         <v>91</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>100</v>
+        <v>162</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="290.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="183">
       <c r="A41" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>102</v>
+        <v>164</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>103</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="409.6">
@@ -4188,288 +4928,288 @@
         <v>72</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>104</v>
+        <v>166</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>105</v>
+        <v>167</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="137.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="409.6">
       <c r="A43" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>104</v>
+        <v>169</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>107</v>
+        <v>170</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="259.5">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="137.25">
       <c r="A44" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>104</v>
+        <v>169</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>109</v>
+        <v>172</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="198">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="259.5">
       <c r="A45" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>104</v>
+        <v>174</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>111</v>
+        <v>175</v>
       </c>
       <c r="D45" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="305.25">
+      <c r="A46" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="409.6">
+      <c r="A47" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D47" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E45" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="259.5">
-      <c r="A46" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="106.5">
-      <c r="A47" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="E47" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="106.5">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="409.6">
       <c r="A48" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>116</v>
+        <v>179</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>119</v>
+        <v>182</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="76.5">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="409.6">
       <c r="A49" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>116</v>
+        <v>179</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>121</v>
+        <v>184</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="259.5">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="409.6">
       <c r="A50" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>123</v>
+        <v>186</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="106.5">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="366">
       <c r="A51" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>116</v>
+        <v>188</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>125</v>
+        <v>189</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="106.5">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="259.5">
       <c r="A52" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>116</v>
+        <v>188</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>127</v>
+        <v>191</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="351">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="259.5">
       <c r="A53" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>88</v>
+        <v>188</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>129</v>
+        <v>193</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="213">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="409.6">
       <c r="A54" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>113</v>
+        <v>188</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>131</v>
+        <v>195</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>44</v>
+        <v>196</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="213">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="259.5">
       <c r="A55" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>113</v>
+        <v>188</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>133</v>
+        <v>198</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>41</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="167.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="366">
       <c r="A56" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="106.5">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="259.5">
       <c r="A57" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>137</v>
+        <v>202</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="275.25">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="366">
       <c r="A58" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>91</v>
+        <v>188</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>139</v>
+        <v>204</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>140</v>
+        <v>8</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>141</v>
+        <v>205</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="409.6">
@@ -4477,19 +5217,19 @@
         <v>72</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>77</v>
+        <v>188</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>142</v>
+        <v>206</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>8</v>
+        <v>196</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="259.5">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="366">
       <c r="A60" s="3" t="s">
         <v>72</v>
       </c>
@@ -4497,30 +5237,30 @@
         <v>88</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>144</v>
+        <v>208</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="183">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="259.5">
       <c r="A61" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>147</v>
+        <v>210</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>148</v>
+        <v>211</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="183">
@@ -4528,50 +5268,50 @@
         <v>72</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>149</v>
+        <v>212</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="198">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="229.5">
       <c r="A63" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>151</v>
+        <v>214</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>41</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="106.5">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="409.6">
       <c r="A64" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>153</v>
+        <v>216</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>154</v>
+        <v>217</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="409.6">
@@ -4579,84 +5319,84 @@
         <v>72</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>155</v>
+        <v>88</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>156</v>
+        <v>218</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>8</v>
+        <v>219</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="409.6">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="366">
       <c r="A66" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>158</v>
+        <v>221</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="229.5">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="409.6">
       <c r="A67" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>91</v>
+        <v>166</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>160</v>
+        <v>223</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="259.5">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="409.6">
       <c r="A68" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>162</v>
+        <v>225</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>44</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="183">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="409.6">
       <c r="A69" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>91</v>
+        <v>166</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>164</v>
+        <v>227</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>165</v>
+        <v>229</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="409.6">
@@ -4667,13 +5407,13 @@
         <v>166</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>168</v>
+        <v>231</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="409.6">
@@ -4681,67 +5421,67 @@
         <v>72</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>170</v>
+        <v>232</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="137.25">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="409.6">
       <c r="A72" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>172</v>
+        <v>234</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" ht="259.5">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="409.6">
       <c r="A73" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>175</v>
+        <v>236</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="305.25">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="409.6">
       <c r="A74" s="3" t="s">
         <v>72</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>177</v>
+        <v>238</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>178</v>
+        <v>239</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="409.6">
@@ -4749,16 +5489,16 @@
         <v>72</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>181</v>
+        <v>241</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="409.6">
@@ -4766,16 +5506,16 @@
         <v>72</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>182</v>
+        <v>242</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>183</v>
+        <v>243</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="409.6">
@@ -4783,492 +5523,50 @@
         <v>72</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>179</v>
+        <v>244</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>184</v>
+        <v>245</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" ht="409.6">
-      <c r="A78" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" ht="366">
-      <c r="A79" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E79" s="5" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" ht="259.5">
-      <c r="A80" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" ht="259.5">
-      <c r="A81" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" ht="409.6">
-      <c r="A82" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" ht="259.5">
-      <c r="A83" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D83" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" ht="366">
-      <c r="A84" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E84" s="5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" ht="259.5">
-      <c r="A85" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" ht="366">
-      <c r="A86" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" ht="409.6">
-      <c r="A87" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" ht="366">
-      <c r="A88" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" ht="259.5">
-      <c r="A89" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="183">
-      <c r="A90" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" ht="229.5">
-      <c r="A91" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" ht="409.6">
-      <c r="A92" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" ht="409.6">
-      <c r="A93" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B93" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" ht="366">
-      <c r="A94" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="409.6">
-      <c r="A95" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" ht="409.6">
-      <c r="A96" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" ht="409.6">
-      <c r="A97" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="D97" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" ht="409.6">
-      <c r="A98" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="D98" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" ht="409.6">
-      <c r="A99" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" ht="409.6">
-      <c r="A100" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="D100" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" ht="409.6">
-      <c r="A101" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="D101" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" ht="409.6">
-      <c r="A102" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D102" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" ht="409.6">
-      <c r="A103" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D103" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" ht="409.6">
-      <c r="A104" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="D104" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E104" s="5" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" ht="409.6">
-      <c r="A105" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="D105" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E105" s="5" t="s">
         <v>246</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87265A3A-5CF8-4421-AD53-CA02C07B0F63}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="5" max="5" width="47.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>